<commit_message>
Updated the schedule and added knockouts
</commit_message>
<xml_diff>
--- a/Entry List 10_40am.xlsx
+++ b/Entry List 10_40am.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\USER-PC\Ravens\Senior Open 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46639DD3-B9C1-4A4A-B62F-3992C6359389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C7BB91-FEFB-4276-85A0-7C75B9BF49A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{264A1161-47FB-460F-8362-5F7BA003EA4C}"/>
+    <workbookView xWindow="1275" yWindow="1035" windowWidth="20370" windowHeight="10905" firstSheet="2" activeTab="2" xr2:uid="{264A1161-47FB-460F-8362-5F7BA003EA4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="213">
   <si>
     <t>Le Roux Strydom</t>
   </si>
@@ -680,9 +680,6 @@
     <t>2nd &amp; Below Group 9</t>
   </si>
   <si>
-    <t>2nd &amp; Below Group 10</t>
-  </si>
-  <si>
     <t>5th &amp; Below Round 32 Match 1</t>
   </si>
   <si>
@@ -693,12 +690,6 @@
   </si>
   <si>
     <t>2nd &amp; Below Round 32 Match 2</t>
-  </si>
-  <si>
-    <t>2nd &amp; Below Round 32 Match 3</t>
-  </si>
-  <si>
-    <t>2nd &amp; Below Round 32 Match 4</t>
   </si>
   <si>
     <t>5th &amp; Below Round 16 Match1</t>
@@ -1937,7 +1928,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>82</v>
@@ -5809,7 +5800,7 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
@@ -6006,7 +5997,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B8" s="29"/>
       <c r="C8" s="29"/>
@@ -6052,22 +6043,22 @@
         <v>99</v>
       </c>
       <c r="E10" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="F10" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="G10" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="H10" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="I10" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="J10" s="17" t="s">
         <v>126</v>
-      </c>
-      <c r="J10" s="17" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
@@ -6077,27 +6068,26 @@
       <c r="B11" s="19">
         <v>0.40625</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="D11" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17" t="s">
+      <c r="F11" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="G11" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="H11" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="I11" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="I11" s="17" t="s">
+      <c r="J11" s="17" t="s">
         <v>126</v>
-      </c>
-      <c r="J11" s="17" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.25">
@@ -6152,7 +6142,9 @@
       <c r="F13" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="G13" s="17"/>
+      <c r="G13" s="17" t="s">
+        <v>143</v>
+      </c>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
       <c r="J13" s="14"/>
@@ -6166,23 +6158,19 @@
         <v>0.625</v>
       </c>
       <c r="C14" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="D14" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="E14" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="F14" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="F14" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="G14" s="16" t="s">
-        <v>210</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>211</v>
-      </c>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
       <c r="K14" s="1"/>
@@ -6195,7 +6183,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>107</v>
@@ -6544,7 +6532,7 @@
     <mergeCell ref="C24:J24"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="C4:J7 C9:J11 D12:J12 C12:C13 D13:G13 C14:H14 C15:J16 G17:J17 C17:F18 C19:J23">
+  <conditionalFormatting sqref="C4:J7 D12:J12 C12:C13 D13:G13 C14:H14 C15:J16 G17:J17 C17:F18 C19:J23 C9:J9 F10:J11 C10:E10 D11:E11">
     <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="5th">
       <formula>NOT(ISERROR(SEARCH("5th",C4)))</formula>
     </cfRule>

</xml_diff>